<commit_message>
test: strengthen financial accounting and risk validation
</commit_message>
<xml_diff>
--- a/models/risk_reporting_model.xlsx
+++ b/models/risk_reporting_model.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R7ff5e96dc288443e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Summary" sheetId="2" r:id="R096a6b61106f4d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VaR" sheetId="3" r:id="R3db548e557f14428"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expected Shortfall" sheetId="4" r:id="R61b4671a74764210"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Income" sheetId="5" r:id="R7459336945074ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Contribution" sheetId="6" r:id="Raea8c1bbef934985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress Tests" sheetId="7" r:id="Rce169f9f1a154789"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yield Curve" sheetId="8" r:id="R9f55c8669ef842f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Attribution" sheetId="9" r:id="Rcdc33f59963947d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="10" r:id="R1f4b0794ec5a4596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions" sheetId="11" r:id="R01ca878c07024c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="12" r:id="R644c8d4283f84331"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Master" sheetId="13" r:id="R1cff00bdcd614653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Data" sheetId="14" r:id="R5ff8916bc6aa45c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Report" sheetId="15" r:id="R1258f56f93b24855"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="16" r:id="R29a22150348d47bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R2be73c38c35746a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Summary" sheetId="2" r:id="Rbbfc9e3829394197"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VaR" sheetId="3" r:id="Re5e9334722124755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expected Shortfall" sheetId="4" r:id="R5e927ece29dc4c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Income" sheetId="5" r:id="R49d92645990847ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Contribution" sheetId="6" r:id="R81dfb3edb02b40f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress Tests" sheetId="7" r:id="R0963f95d7d30456e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yield Curve" sheetId="8" r:id="Rd071504f1c294f20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Attribution" sheetId="9" r:id="Rce0f74aaa3c94aef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="10" r:id="R0558db1b1e2441f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions" sheetId="11" r:id="R978fadbff24c4d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="12" r:id="R11eec6a7f1bd434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Master" sheetId="13" r:id="R1187e6d2b4f94c1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Data" sheetId="14" r:id="Rce389c2a10ce454c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Report" sheetId="15" r:id="Rd377e6fee9044853"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="16" r:id="R5d67f85218074850"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -288,7 +288,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R84d8693b6cb14a50"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R888f670d49894abf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -308,7 +308,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="DataQualityTable" displayName="DataQualityTable" ref="A5:E25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="DataQualityTable" displayName="DataQualityTable" ref="A5:E26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Check"/>
     <x:tableColumn id="2" name="Severity"/>
@@ -802,7 +802,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb32ee0afb6b46b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R100b2cb9ae514e32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -931,7 +931,7 @@
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="7" t="str">
-        <x:v>BOND_TERMS</x:v>
+        <x:v>CASH_RECON</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
         <x:v>PASS</x:v>
@@ -946,7 +946,7 @@
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="7" t="str">
-        <x:v>OPTION_TERMS</x:v>
+        <x:v>BOND_TERMS</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
         <x:v>PASS</x:v>
@@ -961,7 +961,7 @@
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="7" t="str">
-        <x:v>CLASSIFICATION</x:v>
+        <x:v>OPTION_TERMS</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
         <x:v>PASS</x:v>
@@ -976,7 +976,7 @@
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="7" t="str">
-        <x:v>MISSING_PRICE</x:v>
+        <x:v>CLASSIFICATION</x:v>
       </x:c>
       <x:c r="B13" s="7" t="str">
         <x:v>PASS</x:v>
@@ -991,7 +991,7 @@
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="7" t="str">
-        <x:v>STALE_PRICE</x:v>
+        <x:v>MISSING_PRICE</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1006,7 +1006,7 @@
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="7" t="str">
-        <x:v>MISSING_FX</x:v>
+        <x:v>STALE_PRICE</x:v>
       </x:c>
       <x:c r="B15" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1021,7 +1021,7 @@
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="7" t="str">
-        <x:v>STALE_FX</x:v>
+        <x:v>MISSING_FX</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1036,7 +1036,7 @@
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="7" t="str">
-        <x:v>MISSING_FACTOR</x:v>
+        <x:v>STALE_FX</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1051,7 +1051,7 @@
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="7" t="str">
-        <x:v>STALE_FACTOR</x:v>
+        <x:v>MISSING_FACTOR</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1066,7 +1066,7 @@
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="7" t="str">
-        <x:v>CURVE_DATA</x:v>
+        <x:v>STALE_FACTOR</x:v>
       </x:c>
       <x:c r="B19" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1081,7 +1081,7 @@
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="7" t="str">
-        <x:v>FACTOR_CONSISTENCY</x:v>
+        <x:v>CURVE_DATA</x:v>
       </x:c>
       <x:c r="B20" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1096,7 +1096,7 @@
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="7" t="str">
-        <x:v>RETURN_HISTORY</x:v>
+        <x:v>FACTOR_CONSISTENCY</x:v>
       </x:c>
       <x:c r="B21" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1111,7 +1111,7 @@
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="7" t="str">
-        <x:v>OUTLIER</x:v>
+        <x:v>RETURN_HISTORY</x:v>
       </x:c>
       <x:c r="B22" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1126,7 +1126,7 @@
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="7" t="str">
-        <x:v>SHORT_POSITION</x:v>
+        <x:v>OUTLIER</x:v>
       </x:c>
       <x:c r="B23" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1141,7 +1141,7 @@
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="7" t="str">
-        <x:v>POSITION_RECON</x:v>
+        <x:v>SHORT_POSITION</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1156,7 +1156,7 @@
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="7" t="str">
-        <x:v>VALUE_RECON</x:v>
+        <x:v>POSITION_RECON</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
         <x:v>PASS</x:v>
@@ -1169,14 +1169,29 @@
       </x:c>
       <x:c r="E25" s="7" t="str"/>
     </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="7" t="str">
+        <x:v>VALUE_RECON</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="C26" s="7" t="str">
+        <x:v>portfolio</x:v>
+      </x:c>
+      <x:c r="D26" s="7" t="str">
+        <x:v>No exceptions in evaluated scope</x:v>
+      </x:c>
+      <x:c r="E26" s="7" t="str"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="B6:B25">
+  <x:conditionalFormatting sqref="B6:B26">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="WARN"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ebfd8040c7a4cc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c33d6bc3664b4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1532,7 +1547,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a6c51726bae4e82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d55113e920e403c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1910,7 +1925,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3c548d47d704106"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68d182e46c6c422f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2248,7 +2263,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b21202060c84b9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7577e89749d14c80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28304,7 +28319,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d83a070f71c4b1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f1ae1710d184640"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28436,7 +28451,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16787333e00c432d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffdd7d0810b7402c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28583,7 +28598,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R206255f500a347bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9350b7f8a324d52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28714,9 +28729,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86aac4591d274b58"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73b84200f9c24a6f"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf515d8e1377a4e6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca7a7bea32584ae3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28860,7 +28875,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9b4d653d1e446f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08519039a8e341b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28978,7 +28993,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ed0d7120faa4dd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f47b812354e4135"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29122,7 +29137,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6793e4adfec245dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4784d7016b8946d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29390,7 +29405,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R502e4f89b44e4226"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e9554b68f624c03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30010,7 +30025,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44de757463084a0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cfb33318f7d4843"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30214,7 +30229,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R333853b901734e8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a58b8fe059a4105"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30419,7 +30434,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R398346c19a1a41b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bd3142ff052418c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>